<commit_message>
add storages to model input xlsx
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/02_processed/data_case_russia_peak_hour.xlsx
+++ b/01_data/01_input_data/02_processed/data_case_russia_peak_hour.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\02_processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{973F1823-68ED-4EDA-9729-BF851E113DC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F7365A1-953C-4FE5-9A2C-2AEB1ADFBEA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="19380" windowHeight="10170" activeTab="4" xr2:uid="{C00DA6F8-F36F-4C24-9869-33AD338893F6}"/>
   </bookViews>
   <sheets>
     <sheet name="Nodes" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1587" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1860" uniqueCount="120">
   <si>
     <t>Commodities</t>
   </si>
@@ -337,6 +337,69 @@
   </si>
   <si>
     <t>DE_St</t>
+  </si>
+  <si>
+    <t>AT_St</t>
+  </si>
+  <si>
+    <t>BE_St</t>
+  </si>
+  <si>
+    <t>BG_St</t>
+  </si>
+  <si>
+    <t>HR_St</t>
+  </si>
+  <si>
+    <t>CZ_St</t>
+  </si>
+  <si>
+    <t>DK_St</t>
+  </si>
+  <si>
+    <t>FR_St</t>
+  </si>
+  <si>
+    <t>GR_St</t>
+  </si>
+  <si>
+    <t>HU_St</t>
+  </si>
+  <si>
+    <t>IT_St</t>
+  </si>
+  <si>
+    <t>LV_St</t>
+  </si>
+  <si>
+    <t>NL_St</t>
+  </si>
+  <si>
+    <t>PL_St</t>
+  </si>
+  <si>
+    <t>PT_St</t>
+  </si>
+  <si>
+    <t>SK_St</t>
+  </si>
+  <si>
+    <t>SE_St</t>
+  </si>
+  <si>
+    <t>RS_St</t>
+  </si>
+  <si>
+    <t>TR_St</t>
+  </si>
+  <si>
+    <t>UA_St</t>
+  </si>
+  <si>
+    <t>UK_St</t>
+  </si>
+  <si>
+    <t>RO_St</t>
   </si>
 </sst>
 </file>
@@ -694,7 +757,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B0CB446-BDDD-415D-AF22-2CEB1FE45CA5}">
-  <dimension ref="A1:A86"/>
+  <dimension ref="A1:A107"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
@@ -1125,6 +1188,111 @@
     <row r="86" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>98</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A89" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A90" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A91" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A96" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A97" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A98" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A99" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A100" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A101" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A102" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A103" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A104" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A105" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A106" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A107" t="s">
+        <v>118</v>
       </c>
     </row>
   </sheetData>
@@ -1159,7 +1327,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA366CBE-E84C-4E05-9B58-54F3A95EEAB7}">
-  <dimension ref="A1:B143"/>
+  <dimension ref="A1:B164"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
@@ -2304,6 +2472,174 @@
       </c>
       <c r="B143" t="s">
         <v>42</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A144" t="s">
+        <v>99</v>
+      </c>
+      <c r="B144" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A145" t="s">
+        <v>100</v>
+      </c>
+      <c r="B145" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A146" t="s">
+        <v>101</v>
+      </c>
+      <c r="B146" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A147" t="s">
+        <v>102</v>
+      </c>
+      <c r="B147" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A148" t="s">
+        <v>103</v>
+      </c>
+      <c r="B148" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A149" t="s">
+        <v>104</v>
+      </c>
+      <c r="B149" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A150" t="s">
+        <v>105</v>
+      </c>
+      <c r="B150" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A151" t="s">
+        <v>106</v>
+      </c>
+      <c r="B151" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A152" t="s">
+        <v>107</v>
+      </c>
+      <c r="B152" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A153" t="s">
+        <v>108</v>
+      </c>
+      <c r="B153" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A154" t="s">
+        <v>109</v>
+      </c>
+      <c r="B154" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A155" t="s">
+        <v>110</v>
+      </c>
+      <c r="B155" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A156" t="s">
+        <v>111</v>
+      </c>
+      <c r="B156" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A157" t="s">
+        <v>112</v>
+      </c>
+      <c r="B157" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A158" t="s">
+        <v>119</v>
+      </c>
+      <c r="B158" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A159" t="s">
+        <v>113</v>
+      </c>
+      <c r="B159" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A160" t="s">
+        <v>114</v>
+      </c>
+      <c r="B160" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A161" t="s">
+        <v>115</v>
+      </c>
+      <c r="B161" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A162" t="s">
+        <v>116</v>
+      </c>
+      <c r="B162" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A163" t="s">
+        <v>117</v>
+      </c>
+      <c r="B163" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A164" t="s">
+        <v>118</v>
+      </c>
+      <c r="B164" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -2313,7 +2649,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C781A78E-EFEC-4F2E-A496-3B44BD173FD3}">
-  <dimension ref="A1:I287"/>
+  <dimension ref="A1:I329"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
@@ -10636,6 +10972,1224 @@
         <v>1000</v>
       </c>
       <c r="I287">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="288" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A288" t="s">
+        <v>11</v>
+      </c>
+      <c r="B288" t="s">
+        <v>99</v>
+      </c>
+      <c r="C288" t="s">
+        <v>60</v>
+      </c>
+      <c r="D288">
+        <v>100</v>
+      </c>
+      <c r="E288">
+        <v>100</v>
+      </c>
+      <c r="F288">
+        <v>1</v>
+      </c>
+      <c r="G288">
+        <v>10000000</v>
+      </c>
+      <c r="H288">
+        <v>0</v>
+      </c>
+      <c r="I288">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="289" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A289" t="s">
+        <v>11</v>
+      </c>
+      <c r="B289" t="s">
+        <v>100</v>
+      </c>
+      <c r="C289" t="s">
+        <v>16</v>
+      </c>
+      <c r="D289">
+        <v>100</v>
+      </c>
+      <c r="E289">
+        <v>100</v>
+      </c>
+      <c r="F289">
+        <v>1</v>
+      </c>
+      <c r="G289">
+        <v>10000000</v>
+      </c>
+      <c r="H289">
+        <v>0</v>
+      </c>
+      <c r="I289">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="290" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A290" t="s">
+        <v>11</v>
+      </c>
+      <c r="B290" t="s">
+        <v>101</v>
+      </c>
+      <c r="C290" t="s">
+        <v>68</v>
+      </c>
+      <c r="D290">
+        <v>100</v>
+      </c>
+      <c r="E290">
+        <v>100</v>
+      </c>
+      <c r="F290">
+        <v>1</v>
+      </c>
+      <c r="G290">
+        <v>10000000</v>
+      </c>
+      <c r="H290">
+        <v>0</v>
+      </c>
+      <c r="I290">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="291" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A291" t="s">
+        <v>11</v>
+      </c>
+      <c r="B291" t="s">
+        <v>102</v>
+      </c>
+      <c r="C291" t="s">
+        <v>24</v>
+      </c>
+      <c r="D291">
+        <v>100</v>
+      </c>
+      <c r="E291">
+        <v>100</v>
+      </c>
+      <c r="F291">
+        <v>1</v>
+      </c>
+      <c r="G291">
+        <v>10000000</v>
+      </c>
+      <c r="H291">
+        <v>0</v>
+      </c>
+      <c r="I291">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="292" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A292" t="s">
+        <v>11</v>
+      </c>
+      <c r="B292" t="s">
+        <v>103</v>
+      </c>
+      <c r="C292" t="s">
+        <v>62</v>
+      </c>
+      <c r="D292">
+        <v>100</v>
+      </c>
+      <c r="E292">
+        <v>100</v>
+      </c>
+      <c r="F292">
+        <v>1</v>
+      </c>
+      <c r="G292">
+        <v>10000000</v>
+      </c>
+      <c r="H292">
+        <v>0</v>
+      </c>
+      <c r="I292">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="293" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A293" t="s">
+        <v>11</v>
+      </c>
+      <c r="B293" t="s">
+        <v>104</v>
+      </c>
+      <c r="C293" t="s">
+        <v>40</v>
+      </c>
+      <c r="D293">
+        <v>100</v>
+      </c>
+      <c r="E293">
+        <v>100</v>
+      </c>
+      <c r="F293">
+        <v>1</v>
+      </c>
+      <c r="G293">
+        <v>10000000</v>
+      </c>
+      <c r="H293">
+        <v>0</v>
+      </c>
+      <c r="I293">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="294" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A294" t="s">
+        <v>11</v>
+      </c>
+      <c r="B294" t="s">
+        <v>105</v>
+      </c>
+      <c r="C294" t="s">
+        <v>18</v>
+      </c>
+      <c r="D294">
+        <v>100</v>
+      </c>
+      <c r="E294">
+        <v>100</v>
+      </c>
+      <c r="F294">
+        <v>1</v>
+      </c>
+      <c r="G294">
+        <v>10000000</v>
+      </c>
+      <c r="H294">
+        <v>0</v>
+      </c>
+      <c r="I294">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="295" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A295" t="s">
+        <v>11</v>
+      </c>
+      <c r="B295" t="s">
+        <v>106</v>
+      </c>
+      <c r="C295" t="s">
+        <v>20</v>
+      </c>
+      <c r="D295">
+        <v>100</v>
+      </c>
+      <c r="E295">
+        <v>100</v>
+      </c>
+      <c r="F295">
+        <v>1</v>
+      </c>
+      <c r="G295">
+        <v>10000000</v>
+      </c>
+      <c r="H295">
+        <v>0</v>
+      </c>
+      <c r="I295">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="296" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A296" t="s">
+        <v>11</v>
+      </c>
+      <c r="B296" t="s">
+        <v>107</v>
+      </c>
+      <c r="C296" t="s">
+        <v>66</v>
+      </c>
+      <c r="D296">
+        <v>100</v>
+      </c>
+      <c r="E296">
+        <v>100</v>
+      </c>
+      <c r="F296">
+        <v>1</v>
+      </c>
+      <c r="G296">
+        <v>10000000</v>
+      </c>
+      <c r="H296">
+        <v>0</v>
+      </c>
+      <c r="I296">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="297" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A297" t="s">
+        <v>11</v>
+      </c>
+      <c r="B297" t="s">
+        <v>108</v>
+      </c>
+      <c r="C297" t="s">
+        <v>22</v>
+      </c>
+      <c r="D297">
+        <v>100</v>
+      </c>
+      <c r="E297">
+        <v>100</v>
+      </c>
+      <c r="F297">
+        <v>1</v>
+      </c>
+      <c r="G297">
+        <v>10000000</v>
+      </c>
+      <c r="H297">
+        <v>0</v>
+      </c>
+      <c r="I297">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="298" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A298" t="s">
+        <v>11</v>
+      </c>
+      <c r="B298" t="s">
+        <v>109</v>
+      </c>
+      <c r="C298" t="s">
+        <v>72</v>
+      </c>
+      <c r="D298">
+        <v>100</v>
+      </c>
+      <c r="E298">
+        <v>100</v>
+      </c>
+      <c r="F298">
+        <v>1</v>
+      </c>
+      <c r="G298">
+        <v>10000000</v>
+      </c>
+      <c r="H298">
+        <v>0</v>
+      </c>
+      <c r="I298">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="299" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A299" t="s">
+        <v>11</v>
+      </c>
+      <c r="B299" t="s">
+        <v>110</v>
+      </c>
+      <c r="C299" t="s">
+        <v>28</v>
+      </c>
+      <c r="D299">
+        <v>100</v>
+      </c>
+      <c r="E299">
+        <v>100</v>
+      </c>
+      <c r="F299">
+        <v>1</v>
+      </c>
+      <c r="G299">
+        <v>10000000</v>
+      </c>
+      <c r="H299">
+        <v>0</v>
+      </c>
+      <c r="I299">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="300" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A300" t="s">
+        <v>11</v>
+      </c>
+      <c r="B300" t="s">
+        <v>111</v>
+      </c>
+      <c r="C300" t="s">
+        <v>30</v>
+      </c>
+      <c r="D300">
+        <v>100</v>
+      </c>
+      <c r="E300">
+        <v>100</v>
+      </c>
+      <c r="F300">
+        <v>1</v>
+      </c>
+      <c r="G300">
+        <v>10000000</v>
+      </c>
+      <c r="H300">
+        <v>0</v>
+      </c>
+      <c r="I300">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="301" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A301" t="s">
+        <v>11</v>
+      </c>
+      <c r="B301" t="s">
+        <v>112</v>
+      </c>
+      <c r="C301" t="s">
+        <v>32</v>
+      </c>
+      <c r="D301">
+        <v>100</v>
+      </c>
+      <c r="E301">
+        <v>100</v>
+      </c>
+      <c r="F301">
+        <v>1</v>
+      </c>
+      <c r="G301">
+        <v>10000000</v>
+      </c>
+      <c r="H301">
+        <v>0</v>
+      </c>
+      <c r="I301">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="302" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A302" t="s">
+        <v>11</v>
+      </c>
+      <c r="B302" t="s">
+        <v>119</v>
+      </c>
+      <c r="C302" t="s">
+        <v>51</v>
+      </c>
+      <c r="D302">
+        <v>100</v>
+      </c>
+      <c r="E302">
+        <v>100</v>
+      </c>
+      <c r="F302">
+        <v>1</v>
+      </c>
+      <c r="G302">
+        <v>10000000</v>
+      </c>
+      <c r="H302">
+        <v>0</v>
+      </c>
+      <c r="I302">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="303" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A303" t="s">
+        <v>11</v>
+      </c>
+      <c r="B303" t="s">
+        <v>113</v>
+      </c>
+      <c r="C303" t="s">
+        <v>65</v>
+      </c>
+      <c r="D303">
+        <v>100</v>
+      </c>
+      <c r="E303">
+        <v>100</v>
+      </c>
+      <c r="F303">
+        <v>1</v>
+      </c>
+      <c r="G303">
+        <v>10000000</v>
+      </c>
+      <c r="H303">
+        <v>0</v>
+      </c>
+      <c r="I303">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="304" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A304" t="s">
+        <v>11</v>
+      </c>
+      <c r="B304" t="s">
+        <v>114</v>
+      </c>
+      <c r="C304" t="s">
+        <v>79</v>
+      </c>
+      <c r="D304">
+        <v>100</v>
+      </c>
+      <c r="E304">
+        <v>100</v>
+      </c>
+      <c r="F304">
+        <v>1</v>
+      </c>
+      <c r="G304">
+        <v>10000000</v>
+      </c>
+      <c r="H304">
+        <v>0</v>
+      </c>
+      <c r="I304">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="305" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A305" t="s">
+        <v>11</v>
+      </c>
+      <c r="B305" t="s">
+        <v>115</v>
+      </c>
+      <c r="C305" t="s">
+        <v>67</v>
+      </c>
+      <c r="D305">
+        <v>100</v>
+      </c>
+      <c r="E305">
+        <v>100</v>
+      </c>
+      <c r="F305">
+        <v>1</v>
+      </c>
+      <c r="G305">
+        <v>10000000</v>
+      </c>
+      <c r="H305">
+        <v>0</v>
+      </c>
+      <c r="I305">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="306" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A306" t="s">
+        <v>11</v>
+      </c>
+      <c r="B306" t="s">
+        <v>116</v>
+      </c>
+      <c r="C306" t="s">
+        <v>36</v>
+      </c>
+      <c r="D306">
+        <v>100</v>
+      </c>
+      <c r="E306">
+        <v>100</v>
+      </c>
+      <c r="F306">
+        <v>1</v>
+      </c>
+      <c r="G306">
+        <v>10000000</v>
+      </c>
+      <c r="H306">
+        <v>0</v>
+      </c>
+      <c r="I306">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="307" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A307" t="s">
+        <v>11</v>
+      </c>
+      <c r="B307" t="s">
+        <v>117</v>
+      </c>
+      <c r="C307" t="s">
+        <v>58</v>
+      </c>
+      <c r="D307">
+        <v>100</v>
+      </c>
+      <c r="E307">
+        <v>100</v>
+      </c>
+      <c r="F307">
+        <v>1</v>
+      </c>
+      <c r="G307">
+        <v>10000000</v>
+      </c>
+      <c r="H307">
+        <v>0</v>
+      </c>
+      <c r="I307">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="308" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A308" t="s">
+        <v>11</v>
+      </c>
+      <c r="B308" t="s">
+        <v>118</v>
+      </c>
+      <c r="C308" t="s">
+        <v>38</v>
+      </c>
+      <c r="D308">
+        <v>100</v>
+      </c>
+      <c r="E308">
+        <v>100</v>
+      </c>
+      <c r="F308">
+        <v>1</v>
+      </c>
+      <c r="G308">
+        <v>10000000</v>
+      </c>
+      <c r="H308">
+        <v>0</v>
+      </c>
+      <c r="I308">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="309" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A309" t="s">
+        <v>12</v>
+      </c>
+      <c r="B309" t="s">
+        <v>99</v>
+      </c>
+      <c r="C309" t="s">
+        <v>60</v>
+      </c>
+      <c r="D309">
+        <v>10000</v>
+      </c>
+      <c r="E309">
+        <v>10000</v>
+      </c>
+      <c r="F309">
+        <v>100</v>
+      </c>
+      <c r="G309">
+        <v>10000000</v>
+      </c>
+      <c r="H309">
+        <v>1000</v>
+      </c>
+      <c r="I309">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="310" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A310" t="s">
+        <v>12</v>
+      </c>
+      <c r="B310" t="s">
+        <v>100</v>
+      </c>
+      <c r="C310" t="s">
+        <v>16</v>
+      </c>
+      <c r="D310">
+        <v>10000</v>
+      </c>
+      <c r="E310">
+        <v>10000</v>
+      </c>
+      <c r="F310">
+        <v>100</v>
+      </c>
+      <c r="G310">
+        <v>10000000</v>
+      </c>
+      <c r="H310">
+        <v>1000</v>
+      </c>
+      <c r="I310">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="311" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A311" t="s">
+        <v>12</v>
+      </c>
+      <c r="B311" t="s">
+        <v>101</v>
+      </c>
+      <c r="C311" t="s">
+        <v>68</v>
+      </c>
+      <c r="D311">
+        <v>10000</v>
+      </c>
+      <c r="E311">
+        <v>10000</v>
+      </c>
+      <c r="F311">
+        <v>100</v>
+      </c>
+      <c r="G311">
+        <v>10000000</v>
+      </c>
+      <c r="H311">
+        <v>1000</v>
+      </c>
+      <c r="I311">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="312" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A312" t="s">
+        <v>12</v>
+      </c>
+      <c r="B312" t="s">
+        <v>102</v>
+      </c>
+      <c r="C312" t="s">
+        <v>24</v>
+      </c>
+      <c r="D312">
+        <v>10000</v>
+      </c>
+      <c r="E312">
+        <v>10000</v>
+      </c>
+      <c r="F312">
+        <v>100</v>
+      </c>
+      <c r="G312">
+        <v>10000000</v>
+      </c>
+      <c r="H312">
+        <v>1000</v>
+      </c>
+      <c r="I312">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="313" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A313" t="s">
+        <v>12</v>
+      </c>
+      <c r="B313" t="s">
+        <v>103</v>
+      </c>
+      <c r="C313" t="s">
+        <v>62</v>
+      </c>
+      <c r="D313">
+        <v>10000</v>
+      </c>
+      <c r="E313">
+        <v>10000</v>
+      </c>
+      <c r="F313">
+        <v>100</v>
+      </c>
+      <c r="G313">
+        <v>10000000</v>
+      </c>
+      <c r="H313">
+        <v>1000</v>
+      </c>
+      <c r="I313">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="314" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A314" t="s">
+        <v>12</v>
+      </c>
+      <c r="B314" t="s">
+        <v>104</v>
+      </c>
+      <c r="C314" t="s">
+        <v>40</v>
+      </c>
+      <c r="D314">
+        <v>10000</v>
+      </c>
+      <c r="E314">
+        <v>10000</v>
+      </c>
+      <c r="F314">
+        <v>100</v>
+      </c>
+      <c r="G314">
+        <v>10000000</v>
+      </c>
+      <c r="H314">
+        <v>1000</v>
+      </c>
+      <c r="I314">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="315" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A315" t="s">
+        <v>12</v>
+      </c>
+      <c r="B315" t="s">
+        <v>105</v>
+      </c>
+      <c r="C315" t="s">
+        <v>18</v>
+      </c>
+      <c r="D315">
+        <v>10000</v>
+      </c>
+      <c r="E315">
+        <v>10000</v>
+      </c>
+      <c r="F315">
+        <v>100</v>
+      </c>
+      <c r="G315">
+        <v>10000000</v>
+      </c>
+      <c r="H315">
+        <v>1000</v>
+      </c>
+      <c r="I315">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="316" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A316" t="s">
+        <v>12</v>
+      </c>
+      <c r="B316" t="s">
+        <v>106</v>
+      </c>
+      <c r="C316" t="s">
+        <v>20</v>
+      </c>
+      <c r="D316">
+        <v>10000</v>
+      </c>
+      <c r="E316">
+        <v>10000</v>
+      </c>
+      <c r="F316">
+        <v>100</v>
+      </c>
+      <c r="G316">
+        <v>10000000</v>
+      </c>
+      <c r="H316">
+        <v>1000</v>
+      </c>
+      <c r="I316">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="317" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A317" t="s">
+        <v>12</v>
+      </c>
+      <c r="B317" t="s">
+        <v>107</v>
+      </c>
+      <c r="C317" t="s">
+        <v>66</v>
+      </c>
+      <c r="D317">
+        <v>10000</v>
+      </c>
+      <c r="E317">
+        <v>10000</v>
+      </c>
+      <c r="F317">
+        <v>100</v>
+      </c>
+      <c r="G317">
+        <v>10000000</v>
+      </c>
+      <c r="H317">
+        <v>1000</v>
+      </c>
+      <c r="I317">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="318" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A318" t="s">
+        <v>12</v>
+      </c>
+      <c r="B318" t="s">
+        <v>108</v>
+      </c>
+      <c r="C318" t="s">
+        <v>22</v>
+      </c>
+      <c r="D318">
+        <v>10000</v>
+      </c>
+      <c r="E318">
+        <v>10000</v>
+      </c>
+      <c r="F318">
+        <v>100</v>
+      </c>
+      <c r="G318">
+        <v>10000000</v>
+      </c>
+      <c r="H318">
+        <v>1000</v>
+      </c>
+      <c r="I318">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="319" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A319" t="s">
+        <v>12</v>
+      </c>
+      <c r="B319" t="s">
+        <v>109</v>
+      </c>
+      <c r="C319" t="s">
+        <v>72</v>
+      </c>
+      <c r="D319">
+        <v>10000</v>
+      </c>
+      <c r="E319">
+        <v>10000</v>
+      </c>
+      <c r="F319">
+        <v>100</v>
+      </c>
+      <c r="G319">
+        <v>10000000</v>
+      </c>
+      <c r="H319">
+        <v>1000</v>
+      </c>
+      <c r="I319">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="320" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A320" t="s">
+        <v>12</v>
+      </c>
+      <c r="B320" t="s">
+        <v>110</v>
+      </c>
+      <c r="C320" t="s">
+        <v>28</v>
+      </c>
+      <c r="D320">
+        <v>10000</v>
+      </c>
+      <c r="E320">
+        <v>10000</v>
+      </c>
+      <c r="F320">
+        <v>100</v>
+      </c>
+      <c r="G320">
+        <v>10000000</v>
+      </c>
+      <c r="H320">
+        <v>1000</v>
+      </c>
+      <c r="I320">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="321" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A321" t="s">
+        <v>12</v>
+      </c>
+      <c r="B321" t="s">
+        <v>111</v>
+      </c>
+      <c r="C321" t="s">
+        <v>30</v>
+      </c>
+      <c r="D321">
+        <v>10000</v>
+      </c>
+      <c r="E321">
+        <v>10000</v>
+      </c>
+      <c r="F321">
+        <v>100</v>
+      </c>
+      <c r="G321">
+        <v>10000000</v>
+      </c>
+      <c r="H321">
+        <v>1000</v>
+      </c>
+      <c r="I321">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="322" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A322" t="s">
+        <v>12</v>
+      </c>
+      <c r="B322" t="s">
+        <v>112</v>
+      </c>
+      <c r="C322" t="s">
+        <v>32</v>
+      </c>
+      <c r="D322">
+        <v>10000</v>
+      </c>
+      <c r="E322">
+        <v>10000</v>
+      </c>
+      <c r="F322">
+        <v>100</v>
+      </c>
+      <c r="G322">
+        <v>10000000</v>
+      </c>
+      <c r="H322">
+        <v>1000</v>
+      </c>
+      <c r="I322">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="323" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A323" t="s">
+        <v>12</v>
+      </c>
+      <c r="B323" t="s">
+        <v>119</v>
+      </c>
+      <c r="C323" t="s">
+        <v>51</v>
+      </c>
+      <c r="D323">
+        <v>10000</v>
+      </c>
+      <c r="E323">
+        <v>10000</v>
+      </c>
+      <c r="F323">
+        <v>100</v>
+      </c>
+      <c r="G323">
+        <v>10000000</v>
+      </c>
+      <c r="H323">
+        <v>1000</v>
+      </c>
+      <c r="I323">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="324" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A324" t="s">
+        <v>12</v>
+      </c>
+      <c r="B324" t="s">
+        <v>113</v>
+      </c>
+      <c r="C324" t="s">
+        <v>65</v>
+      </c>
+      <c r="D324">
+        <v>10000</v>
+      </c>
+      <c r="E324">
+        <v>10000</v>
+      </c>
+      <c r="F324">
+        <v>100</v>
+      </c>
+      <c r="G324">
+        <v>10000000</v>
+      </c>
+      <c r="H324">
+        <v>1000</v>
+      </c>
+      <c r="I324">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="325" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A325" t="s">
+        <v>12</v>
+      </c>
+      <c r="B325" t="s">
+        <v>114</v>
+      </c>
+      <c r="C325" t="s">
+        <v>79</v>
+      </c>
+      <c r="D325">
+        <v>10000</v>
+      </c>
+      <c r="E325">
+        <v>10000</v>
+      </c>
+      <c r="F325">
+        <v>100</v>
+      </c>
+      <c r="G325">
+        <v>10000000</v>
+      </c>
+      <c r="H325">
+        <v>1000</v>
+      </c>
+      <c r="I325">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="326" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A326" t="s">
+        <v>12</v>
+      </c>
+      <c r="B326" t="s">
+        <v>115</v>
+      </c>
+      <c r="C326" t="s">
+        <v>67</v>
+      </c>
+      <c r="D326">
+        <v>10000</v>
+      </c>
+      <c r="E326">
+        <v>10000</v>
+      </c>
+      <c r="F326">
+        <v>100</v>
+      </c>
+      <c r="G326">
+        <v>10000000</v>
+      </c>
+      <c r="H326">
+        <v>1000</v>
+      </c>
+      <c r="I326">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="327" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A327" t="s">
+        <v>12</v>
+      </c>
+      <c r="B327" t="s">
+        <v>116</v>
+      </c>
+      <c r="C327" t="s">
+        <v>36</v>
+      </c>
+      <c r="D327">
+        <v>10000</v>
+      </c>
+      <c r="E327">
+        <v>10000</v>
+      </c>
+      <c r="F327">
+        <v>100</v>
+      </c>
+      <c r="G327">
+        <v>10000000</v>
+      </c>
+      <c r="H327">
+        <v>1000</v>
+      </c>
+      <c r="I327">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="328" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A328" t="s">
+        <v>12</v>
+      </c>
+      <c r="B328" t="s">
+        <v>117</v>
+      </c>
+      <c r="C328" t="s">
+        <v>58</v>
+      </c>
+      <c r="D328">
+        <v>10000</v>
+      </c>
+      <c r="E328">
+        <v>10000</v>
+      </c>
+      <c r="F328">
+        <v>100</v>
+      </c>
+      <c r="G328">
+        <v>10000000</v>
+      </c>
+      <c r="H328">
+        <v>1000</v>
+      </c>
+      <c r="I328">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="329" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A329" t="s">
+        <v>12</v>
+      </c>
+      <c r="B329" t="s">
+        <v>118</v>
+      </c>
+      <c r="C329" t="s">
+        <v>38</v>
+      </c>
+      <c r="D329">
+        <v>10000</v>
+      </c>
+      <c r="E329">
+        <v>10000</v>
+      </c>
+      <c r="F329">
+        <v>100</v>
+      </c>
+      <c r="G329">
+        <v>10000000</v>
+      </c>
+      <c r="H329">
+        <v>1000</v>
+      </c>
+      <c r="I329">
         <v>1</v>
       </c>
     </row>
@@ -10647,7 +12201,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C68B577B-1347-43AB-A697-F4519763B965}">
-  <dimension ref="A1:C172"/>
+  <dimension ref="A1:C214"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -12542,6 +14096,468 @@
         <v>0</v>
       </c>
     </row>
+    <row r="173" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A173" t="s">
+        <v>11</v>
+      </c>
+      <c r="B173" t="s">
+        <v>99</v>
+      </c>
+      <c r="C173">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="174" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A174" t="s">
+        <v>11</v>
+      </c>
+      <c r="B174" t="s">
+        <v>100</v>
+      </c>
+      <c r="C174">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="175" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A175" t="s">
+        <v>11</v>
+      </c>
+      <c r="B175" t="s">
+        <v>101</v>
+      </c>
+      <c r="C175">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="176" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A176" t="s">
+        <v>11</v>
+      </c>
+      <c r="B176" t="s">
+        <v>102</v>
+      </c>
+      <c r="C176">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="177" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A177" t="s">
+        <v>11</v>
+      </c>
+      <c r="B177" t="s">
+        <v>103</v>
+      </c>
+      <c r="C177">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="178" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A178" t="s">
+        <v>11</v>
+      </c>
+      <c r="B178" t="s">
+        <v>104</v>
+      </c>
+      <c r="C178">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="179" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A179" t="s">
+        <v>11</v>
+      </c>
+      <c r="B179" t="s">
+        <v>105</v>
+      </c>
+      <c r="C179">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="180" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A180" t="s">
+        <v>11</v>
+      </c>
+      <c r="B180" t="s">
+        <v>106</v>
+      </c>
+      <c r="C180">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="181" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A181" t="s">
+        <v>11</v>
+      </c>
+      <c r="B181" t="s">
+        <v>107</v>
+      </c>
+      <c r="C181">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="182" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A182" t="s">
+        <v>11</v>
+      </c>
+      <c r="B182" t="s">
+        <v>108</v>
+      </c>
+      <c r="C182">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="183" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A183" t="s">
+        <v>11</v>
+      </c>
+      <c r="B183" t="s">
+        <v>109</v>
+      </c>
+      <c r="C183">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="184" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A184" t="s">
+        <v>11</v>
+      </c>
+      <c r="B184" t="s">
+        <v>110</v>
+      </c>
+      <c r="C184">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="185" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A185" t="s">
+        <v>11</v>
+      </c>
+      <c r="B185" t="s">
+        <v>111</v>
+      </c>
+      <c r="C185">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="186" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A186" t="s">
+        <v>11</v>
+      </c>
+      <c r="B186" t="s">
+        <v>112</v>
+      </c>
+      <c r="C186">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="187" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A187" t="s">
+        <v>11</v>
+      </c>
+      <c r="B187" t="s">
+        <v>119</v>
+      </c>
+      <c r="C187">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="188" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A188" t="s">
+        <v>11</v>
+      </c>
+      <c r="B188" t="s">
+        <v>113</v>
+      </c>
+      <c r="C188">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="189" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A189" t="s">
+        <v>11</v>
+      </c>
+      <c r="B189" t="s">
+        <v>114</v>
+      </c>
+      <c r="C189">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="190" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A190" t="s">
+        <v>11</v>
+      </c>
+      <c r="B190" t="s">
+        <v>115</v>
+      </c>
+      <c r="C190">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="191" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A191" t="s">
+        <v>11</v>
+      </c>
+      <c r="B191" t="s">
+        <v>116</v>
+      </c>
+      <c r="C191">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="192" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A192" t="s">
+        <v>11</v>
+      </c>
+      <c r="B192" t="s">
+        <v>117</v>
+      </c>
+      <c r="C192">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="193" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A193" t="s">
+        <v>11</v>
+      </c>
+      <c r="B193" t="s">
+        <v>118</v>
+      </c>
+      <c r="C193">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="194" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A194" t="s">
+        <v>12</v>
+      </c>
+      <c r="B194" t="s">
+        <v>99</v>
+      </c>
+      <c r="C194">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="195" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A195" t="s">
+        <v>12</v>
+      </c>
+      <c r="B195" t="s">
+        <v>100</v>
+      </c>
+      <c r="C195">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="196" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A196" t="s">
+        <v>12</v>
+      </c>
+      <c r="B196" t="s">
+        <v>101</v>
+      </c>
+      <c r="C196">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="197" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A197" t="s">
+        <v>12</v>
+      </c>
+      <c r="B197" t="s">
+        <v>102</v>
+      </c>
+      <c r="C197">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="198" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A198" t="s">
+        <v>12</v>
+      </c>
+      <c r="B198" t="s">
+        <v>103</v>
+      </c>
+      <c r="C198">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="199" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A199" t="s">
+        <v>12</v>
+      </c>
+      <c r="B199" t="s">
+        <v>104</v>
+      </c>
+      <c r="C199">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="200" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A200" t="s">
+        <v>12</v>
+      </c>
+      <c r="B200" t="s">
+        <v>105</v>
+      </c>
+      <c r="C200">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="201" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A201" t="s">
+        <v>12</v>
+      </c>
+      <c r="B201" t="s">
+        <v>106</v>
+      </c>
+      <c r="C201">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="202" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A202" t="s">
+        <v>12</v>
+      </c>
+      <c r="B202" t="s">
+        <v>107</v>
+      </c>
+      <c r="C202">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="203" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A203" t="s">
+        <v>12</v>
+      </c>
+      <c r="B203" t="s">
+        <v>108</v>
+      </c>
+      <c r="C203">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="204" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A204" t="s">
+        <v>12</v>
+      </c>
+      <c r="B204" t="s">
+        <v>109</v>
+      </c>
+      <c r="C204">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="205" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A205" t="s">
+        <v>12</v>
+      </c>
+      <c r="B205" t="s">
+        <v>110</v>
+      </c>
+      <c r="C205">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="206" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A206" t="s">
+        <v>12</v>
+      </c>
+      <c r="B206" t="s">
+        <v>111</v>
+      </c>
+      <c r="C206">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="207" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A207" t="s">
+        <v>12</v>
+      </c>
+      <c r="B207" t="s">
+        <v>112</v>
+      </c>
+      <c r="C207">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="208" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A208" t="s">
+        <v>12</v>
+      </c>
+      <c r="B208" t="s">
+        <v>119</v>
+      </c>
+      <c r="C208">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="209" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A209" t="s">
+        <v>12</v>
+      </c>
+      <c r="B209" t="s">
+        <v>113</v>
+      </c>
+      <c r="C209">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="210" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A210" t="s">
+        <v>12</v>
+      </c>
+      <c r="B210" t="s">
+        <v>114</v>
+      </c>
+      <c r="C210">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="211" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A211" t="s">
+        <v>12</v>
+      </c>
+      <c r="B211" t="s">
+        <v>115</v>
+      </c>
+      <c r="C211">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="212" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A212" t="s">
+        <v>12</v>
+      </c>
+      <c r="B212" t="s">
+        <v>116</v>
+      </c>
+      <c r="C212">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="213" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A213" t="s">
+        <v>12</v>
+      </c>
+      <c r="B213" t="s">
+        <v>117</v>
+      </c>
+      <c r="C213">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="214" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A214" t="s">
+        <v>12</v>
+      </c>
+      <c r="B214" t="s">
+        <v>118</v>
+      </c>
+      <c r="C214">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>